<commit_message>
Propuestas actualizadas nuevos desarrollos
</commit_message>
<xml_diff>
--- a/documentos/RQM Aprobacion Ajustes OC/Matriz de Pruebas.xlsx
+++ b/documentos/RQM Aprobacion Ajustes OC/Matriz de Pruebas.xlsx
@@ -9,13 +9,14 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="450" windowWidth="20400" windowHeight="7890" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="900" windowWidth="0" windowHeight="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Configuracion Tolerancia" sheetId="1" r:id="rId1"/>
     <sheet name="Ordenes de Compra" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1082,11 +1083,11 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1379,12 +1380,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
     </row>
     <row r="3" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -1928,13 +1929,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="3" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -2062,13 +2063,13 @@
       </c>
     </row>
     <row r="11" spans="1:6" ht="21" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
     </row>
     <row r="13" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
@@ -2117,7 +2118,7 @@
       <c r="D15" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="E15" s="8"/>
+      <c r="E15" s="7"/>
     </row>
     <row r="16" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -2132,7 +2133,7 @@
       <c r="D16" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="E16" s="8"/>
+      <c r="E16" s="7"/>
     </row>
     <row r="17" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
@@ -2147,7 +2148,7 @@
       <c r="D17" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="E17" s="8"/>
+      <c r="E17" s="7"/>
     </row>
     <row r="18" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
@@ -2162,7 +2163,7 @@
       <c r="D18" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="E18" s="8"/>
+      <c r="E18" s="7"/>
     </row>
     <row r="19" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
@@ -2182,13 +2183,13 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
     </row>
     <row r="23" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
@@ -2310,16 +2311,16 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E30" s="8"/>
+      <c r="E30" s="7"/>
     </row>
     <row r="31" spans="1:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="A31" s="7" t="s">
+      <c r="A31" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
@@ -2390,13 +2391,13 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="A38" s="7" t="s">
+      <c r="A38" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="B38" s="7"/>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
-      <c r="E38" s="7"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
     </row>
     <row r="40" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
@@ -2501,13 +2502,13 @@
       </c>
     </row>
     <row r="47" spans="1:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="A47" s="7" t="s">
+      <c r="A47" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="B47" s="7"/>
-      <c r="C47" s="7"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="7"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="8"/>
     </row>
     <row r="49" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
@@ -2663,13 +2664,13 @@
       </c>
     </row>
     <row r="59" spans="1:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="A59" s="7" t="s">
+      <c r="A59" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="B59" s="7"/>
-      <c r="C59" s="7"/>
-      <c r="D59" s="7"/>
-      <c r="E59" s="7"/>
+      <c r="B59" s="8"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="8"/>
+      <c r="E59" s="8"/>
     </row>
     <row r="61" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
@@ -2808,13 +2809,13 @@
       </c>
     </row>
     <row r="70" spans="1:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="A70" s="7" t="s">
+      <c r="A70" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="B70" s="7"/>
-      <c r="C70" s="7"/>
-      <c r="D70" s="7"/>
-      <c r="E70" s="7"/>
+      <c r="B70" s="8"/>
+      <c r="C70" s="8"/>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8"/>
     </row>
     <row r="72" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
@@ -2880,7 +2881,7 @@
       <c r="D75" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="E75" s="8"/>
+      <c r="E75" s="7"/>
     </row>
     <row r="76" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
@@ -2895,16 +2896,16 @@
       <c r="D76" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="E76" s="8"/>
+      <c r="E76" s="7"/>
     </row>
     <row r="78" spans="1:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="A78" s="7" t="s">
+      <c r="A78" s="8" t="s">
         <v>270</v>
       </c>
-      <c r="B78" s="7"/>
-      <c r="C78" s="7"/>
-      <c r="D78" s="7"/>
-      <c r="E78" s="7"/>
+      <c r="B78" s="8"/>
+      <c r="C78" s="8"/>
+      <c r="D78" s="8"/>
+      <c r="E78" s="8"/>
     </row>
     <row r="80" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">

</xml_diff>